<commit_message>
CooLinens sheets: re-base Batch 1 at the launch price (Vine row)
Queen 87.99, King 93.99, Cal King 95.99, Full 74.99, Twin 69.99 per the
14 Oct launch price decision. Ceilings, bids, top of search steps and
budgets recalculate; 29 cells change in the upload file (gate ALL PASS,
64 of 64 lines reconciled). Batch 1 spend about 189 a day, budgets 486,
expected ACoS 39.2%. Fixes the Campaigns objective label on cooling
sheets queen size, the CooLinens fabric (CooLoom, 16 inch pocket) and
review count, competitor price comparisons and the page text.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJUn53DicDcqHAh1hw7jdv
</commit_message>
<xml_diff>
--- a/deliverables/coolinens-cooling-sheets/bulk/COOLINENS_Cooling_Sheets_4PC_Batch1_Launch_Bulk_20261015.xlsx
+++ b/deliverables/coolinens-cooling-sheets/bulk/COOLINENS_Cooling_Sheets_4PC_Batch1_Launch_Bulk_20261015.xlsx
@@ -743,7 +743,7 @@
         </is>
       </c>
       <c r="U2" t="n">
-        <v>66</v>
+        <v>81</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -832,7 +832,7 @@
         </is>
       </c>
       <c r="Z4" t="n">
-        <v>1.15</v>
+        <v>1.41</v>
       </c>
     </row>
     <row r="5">
@@ -947,7 +947,7 @@
         </is>
       </c>
       <c r="AB7" t="n">
-        <v>1.15</v>
+        <v>1.41</v>
       </c>
       <c r="AC7" t="inlineStr">
         <is>
@@ -1092,7 +1092,7 @@
         </is>
       </c>
       <c r="Z10" t="n">
-        <v>2.62</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="11">
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="AB12" t="n">
-        <v>2.62</v>
+        <v>2.7</v>
       </c>
       <c r="AC12" t="inlineStr">
         <is>
@@ -1224,7 +1224,7 @@
         </is>
       </c>
       <c r="U13" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="AG13" t="inlineStr">
         <is>
@@ -1271,7 +1271,7 @@
         </is>
       </c>
       <c r="AI14" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
     </row>
     <row r="15">
@@ -1534,7 +1534,7 @@
         </is>
       </c>
       <c r="Z20" t="n">
-        <v>2.72</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="21">
@@ -1610,7 +1610,7 @@
         </is>
       </c>
       <c r="AB22" t="n">
-        <v>2.72</v>
+        <v>3.34</v>
       </c>
       <c r="AC22" t="inlineStr">
         <is>
@@ -1713,7 +1713,7 @@
         </is>
       </c>
       <c r="AI24" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
     </row>
     <row r="25">
@@ -1934,7 +1934,7 @@
         </is>
       </c>
       <c r="AI29" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
     </row>
     <row r="30">
@@ -2155,7 +2155,7 @@
         </is>
       </c>
       <c r="AI34" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
     </row>
     <row r="35">
@@ -2597,7 +2597,7 @@
         </is>
       </c>
       <c r="Z44" t="n">
-        <v>1.66</v>
+        <v>2.03</v>
       </c>
     </row>
     <row r="45">
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="AB46" t="n">
-        <v>1.66</v>
+        <v>2.03</v>
       </c>
       <c r="AC46" t="inlineStr">
         <is>
@@ -2776,7 +2776,7 @@
         </is>
       </c>
       <c r="Z48" t="n">
-        <v>2.88</v>
+        <v>3.11</v>
       </c>
     </row>
     <row r="49">
@@ -2852,7 +2852,7 @@
         </is>
       </c>
       <c r="AB50" t="n">
-        <v>2.88</v>
+        <v>3.11</v>
       </c>
       <c r="AC50" t="inlineStr">
         <is>
@@ -4745,7 +4745,7 @@
         </is>
       </c>
       <c r="Z92" t="n">
-        <v>2.05</v>
+        <v>2.17</v>
       </c>
     </row>
     <row r="93">
@@ -4821,7 +4821,7 @@
         </is>
       </c>
       <c r="AB94" t="n">
-        <v>2.05</v>
+        <v>2.17</v>
       </c>
       <c r="AC94" t="inlineStr">
         <is>
@@ -5461,7 +5461,7 @@
         </is>
       </c>
       <c r="Z108" t="n">
-        <v>2.86</v>
+        <v>2.89</v>
       </c>
     </row>
     <row r="109">
@@ -5537,7 +5537,7 @@
         </is>
       </c>
       <c r="AB110" t="n">
-        <v>2.86</v>
+        <v>2.89</v>
       </c>
       <c r="AC110" t="inlineStr">
         <is>
@@ -8164,7 +8164,7 @@
         </is>
       </c>
       <c r="Z169" t="n">
-        <v>2.13</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="170">
@@ -8240,7 +8240,7 @@
         </is>
       </c>
       <c r="AB171" t="n">
-        <v>2.13</v>
+        <v>2.7</v>
       </c>
       <c r="AC171" t="inlineStr">
         <is>
@@ -8292,7 +8292,7 @@
         </is>
       </c>
       <c r="Z172" t="n">
-        <v>2.13</v>
+        <v>2.19</v>
       </c>
     </row>
     <row r="173">
@@ -8368,7 +8368,7 @@
         </is>
       </c>
       <c r="AB174" t="n">
-        <v>2.13</v>
+        <v>2.19</v>
       </c>
       <c r="AC174" t="inlineStr">
         <is>
@@ -8867,7 +8867,7 @@
         </is>
       </c>
       <c r="AB185" t="n">
-        <v>2.86</v>
+        <v>2.9</v>
       </c>
       <c r="AC185" t="inlineStr">
         <is>
@@ -9403,7 +9403,7 @@
         </is>
       </c>
       <c r="AB197" t="n">
-        <v>2.41</v>
+        <v>2.54</v>
       </c>
       <c r="AJ197" t="inlineStr">
         <is>
@@ -9487,7 +9487,7 @@
         </is>
       </c>
       <c r="AB199" t="n">
-        <v>2.41</v>
+        <v>2.62</v>
       </c>
       <c r="AJ199" t="inlineStr">
         <is>
@@ -9571,7 +9571,7 @@
         </is>
       </c>
       <c r="AB201" t="n">
-        <v>2.41</v>
+        <v>2.95</v>
       </c>
       <c r="AJ201" t="inlineStr">
         <is>
@@ -9778,7 +9778,7 @@
         </is>
       </c>
       <c r="AB206" t="n">
-        <v>2.39</v>
+        <v>3</v>
       </c>
       <c r="AJ206" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
CooLinens sheets: Batch 1 campaigns uploaded paused for the 10 AM ET switch-on
All 40 campaigns set to paused in the Batch 1 bulk (ad groups, keywords and
targets stay enabled) so the file can go up ahead of the Featured Offer check.
Bulk_Reconciliation start-date note updated. Validator ALL PASS; recalc 0 errors.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJUn53DicDcqHAh1hw7jdv
</commit_message>
<xml_diff>
--- a/deliverables/coolinens-cooling-sheets/bulk/COOLINENS_Cooling_Sheets_4PC_Batch1_Launch_Bulk_20261015.xlsx
+++ b/deliverables/coolinens-cooling-sheets/bulk/COOLINENS_Cooling_Sheets_4PC_Batch1_Launch_Bulk_20261015.xlsx
@@ -739,7 +739,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U2" t="n">
@@ -999,7 +999,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U8" t="n">
@@ -1220,7 +1220,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U13" t="n">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U18" t="n">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U23" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U28" t="n">
@@ -2104,7 +2104,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U33" t="n">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U38" t="n">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U42" t="n">
@@ -2725,7 +2725,7 @@
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U47" t="n">
@@ -2904,7 +2904,7 @@
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U51" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U55" t="n">
@@ -3262,7 +3262,7 @@
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U59" t="n">
@@ -3441,7 +3441,7 @@
       </c>
       <c r="R63" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U63" t="n">
@@ -3620,7 +3620,7 @@
       </c>
       <c r="R67" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U67" t="n">
@@ -3799,7 +3799,7 @@
       </c>
       <c r="R71" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U71" t="n">
@@ -3978,7 +3978,7 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U75" t="n">
@@ -4157,7 +4157,7 @@
       </c>
       <c r="R79" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U79" t="n">
@@ -4336,7 +4336,7 @@
       </c>
       <c r="R83" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U83" t="n">
@@ -4515,7 +4515,7 @@
       </c>
       <c r="R87" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U87" t="n">
@@ -4694,7 +4694,7 @@
       </c>
       <c r="R91" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U91" t="n">
@@ -4873,7 +4873,7 @@
       </c>
       <c r="R95" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U95" t="n">
@@ -5052,7 +5052,7 @@
       </c>
       <c r="R99" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U99" t="n">
@@ -5231,7 +5231,7 @@
       </c>
       <c r="R103" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U103" t="n">
@@ -5410,7 +5410,7 @@
       </c>
       <c r="R107" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U107" t="n">
@@ -5589,7 +5589,7 @@
       </c>
       <c r="R111" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U111" t="n">
@@ -5768,7 +5768,7 @@
       </c>
       <c r="R115" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U115" t="n">
@@ -5947,7 +5947,7 @@
       </c>
       <c r="R119" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U119" t="n">
@@ -6126,7 +6126,7 @@
       </c>
       <c r="R123" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U123" t="n">
@@ -6305,7 +6305,7 @@
       </c>
       <c r="R127" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U127" t="n">
@@ -6484,7 +6484,7 @@
       </c>
       <c r="R131" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U131" t="n">
@@ -6663,7 +6663,7 @@
       </c>
       <c r="R135" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U135" t="n">
@@ -6842,7 +6842,7 @@
       </c>
       <c r="R139" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U139" t="n">
@@ -7021,7 +7021,7 @@
       </c>
       <c r="R143" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U143" t="n">
@@ -7328,7 +7328,7 @@
       </c>
       <c r="R150" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U150" t="n">
@@ -7682,7 +7682,7 @@
       </c>
       <c r="R158" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U158" t="n">
@@ -8420,7 +8420,7 @@
       </c>
       <c r="R175" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U175" t="n">
@@ -8646,7 +8646,7 @@
       </c>
       <c r="R180" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U180" t="n">
@@ -8966,7 +8966,7 @@
       </c>
       <c r="R187" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U187" t="n">
@@ -9192,7 +9192,7 @@
       </c>
       <c r="R192" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>paused</t>
         </is>
       </c>
       <c r="U192" t="n">

</xml_diff>